<commit_message>
Fix some WG words format
</commit_message>
<xml_diff>
--- a/data/2026_S_M_WG.xlsx
+++ b/data/2026_S_M_WG.xlsx
@@ -5,16 +5,18 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f525d8bd7cc13637/채아_SALT/2026_Spring/Geography/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project\word-tester\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="8_{3A2E5DF6-C3AA-4270-894F-EC23CA0760DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C26DD1A3-0DFE-4D22-A3CB-AB390B24C8FB}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D5020C5-0396-45E6-89CF-E3C386E9A4DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D44E7B26-D9FB-41A9-A2D1-87DDBB0C4DFE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{D44E7B26-D9FB-41A9-A2D1-87DDBB0C4DFE}"/>
   </bookViews>
   <sheets>
-    <sheet name="English" sheetId="2" r:id="rId1"/>
-    <sheet name="Korean" sheetId="1" r:id="rId2"/>
+    <sheet name="N&amp;S Europe" sheetId="2" r:id="rId1"/>
+    <sheet name="East Asia" sheetId="3" r:id="rId2"/>
+    <sheet name="Southeast Asia" sheetId="4" r:id="rId3"/>
+    <sheet name="Korean" sheetId="1" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="152">
   <si>
     <t>지역 (Chapter)</t>
   </si>
@@ -727,171 +729,90 @@
     <t>a period of artistic and intellectual activity</t>
   </si>
   <si>
-    <t>Homogeneous</t>
-  </si>
-  <si>
     <t>similar</t>
   </si>
   <si>
-    <t>Dialect</t>
-  </si>
-  <si>
     <t>a regional variety of a language with unique features, such as vocabulary, grammar, or pronunciation</t>
   </si>
   <si>
-    <t>Welfare capitalism</t>
-  </si>
-  <si>
     <t>a system in which the government uses tax money to provide services, such as health care and education, to all citizens</t>
   </si>
   <si>
-    <t>Recession</t>
-  </si>
-  <si>
     <t>a period of slow economic growth or decline</t>
   </si>
   <si>
     <t>East Asia</t>
   </si>
   <si>
-    <t>De facto</t>
-  </si>
-  <si>
     <t>actually; in reality</t>
   </si>
   <si>
-    <t>Archipelago</t>
-  </si>
-  <si>
     <t>a group of islands</t>
   </si>
   <si>
-    <t>Tsunami</t>
-  </si>
-  <si>
     <t>a giant ocean wave caused by an earthquake under the ocean floor</t>
   </si>
   <si>
-    <t>Loess</t>
-  </si>
-  <si>
     <t>a fine-grained, fertile soil deposited by the wind</t>
   </si>
   <si>
-    <t>Dynasty</t>
-  </si>
-  <si>
     <t>a line of rulers from a single family that holds power for a long time</t>
   </si>
   <si>
-    <t>Shogun</t>
-  </si>
-  <si>
     <t>a military leader who ruled Japan in early times</t>
   </si>
   <si>
-    <t>Samurai</t>
-  </si>
-  <si>
     <t>a powerful, land-owning warrior in Japan</t>
   </si>
   <si>
-    <t>Sphere of influence</t>
-  </si>
-  <si>
     <t>an area of a country where a single foreign power has been granted exclusive trading rights</t>
   </si>
   <si>
-    <t>Communism</t>
-  </si>
-  <si>
     <t>a system of government in which the government controls the ways of producing goods</t>
   </si>
   <si>
-    <t>Urbanization</t>
-  </si>
-  <si>
     <t>growth of a city into nearby areas</t>
   </si>
   <si>
-    <t>Megalopolis</t>
-  </si>
-  <si>
     <t>a huge city or cluster of cities with an extremely large population</t>
   </si>
   <si>
-    <t>Trade deficit</t>
-  </si>
-  <si>
     <t>occurs when the value of a country's imports is higher than the value of its exports</t>
   </si>
   <si>
-    <t>Trade surplus</t>
-  </si>
-  <si>
     <t>occurs when the value of a country's exports is higher than the value of its imports</t>
   </si>
   <si>
     <t>Southeast Asia</t>
   </si>
   <si>
-    <t>Insular</t>
-  </si>
-  <si>
     <t>an area consisting of islands</t>
   </si>
   <si>
-    <t>Flora</t>
-  </si>
-  <si>
     <t>plant life</t>
   </si>
   <si>
-    <t>Fauna</t>
-  </si>
-  <si>
     <t>animal life</t>
   </si>
   <si>
-    <t>Endemic</t>
-  </si>
-  <si>
     <t>found only in one place or region</t>
   </si>
   <si>
-    <t>Sultan</t>
-  </si>
-  <si>
     <t>a king</t>
   </si>
   <si>
-    <t>Plantation</t>
-  </si>
-  <si>
     <t>a large farm on which a single crop is grown for export</t>
   </si>
   <si>
-    <t>Absolute monarchy</t>
-  </si>
-  <si>
     <t>a government in which one ruler has total control</t>
   </si>
   <si>
-    <t>Constitutional monarchy</t>
-  </si>
-  <si>
     <t>a government in which a ruler must follow a constitution and laws</t>
   </si>
   <si>
-    <t>Primate city</t>
-  </si>
-  <si>
     <t>a city so large and important that it dominates the rest of the country</t>
   </si>
   <si>
-    <t>Minority</t>
-  </si>
-  <si>
     <t>small ethnic group within a country</t>
   </si>
   <si>
@@ -901,63 +822,12 @@
     <t>the area bordering the Pacific Ocean</t>
   </si>
   <si>
-    <t>Subsistence farming</t>
-  </si>
-  <si>
     <t>type of farming in which only enough food is grown to feed one's family</t>
   </si>
   <si>
-    <t>Ecotourism</t>
-  </si>
-  <si>
     <t>touring natural environments such as rain forests and coral reefs</t>
   </si>
   <si>
-    <t>Archipelago
-City-state
-Communism
-De facto
-Dialect
-Dynasty
-Fjord
-Glaciation
-Homogeneous
-Loess
-Longship
-Megalopolis
-Pagan
-Recession
-Renaissance
-Samurai
-Scrubland
-Shogun
-Sphere of influence
-Trawler
-Tsunami
-Tundra
-Urbanization
-Welfare capitalism</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Absolute monarchy
-Constitutional monarchy
-Ecotourism
-Endemic
-Fauna
-Flora
-Insular
-Minority
-Pacific Rim
-Plantation
-Primate city
-Subsistence farming
-Sultan
-Trade deficit
-Trade surplus</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>glaciation</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -987,6 +857,122 @@
   </si>
   <si>
     <t>pagan</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>homogeneous</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>dialect</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>welfare capitalism</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>recession</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>de facto</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>archipelago</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>tsunami</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>loess</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>dynasty</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>shogun</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>samurai</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>sphere of influence</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>communism</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>urbanization</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>megalopolis</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>trade deficit</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>trade surplus</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>insular</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>flora</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>fauna</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>endemic</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>sultan</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>plantation</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>absolute monarchy</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>constitutional monarchy</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>primate city</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>minority</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>subsistence farming</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ecotourism</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -994,7 +980,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1016,14 +1002,6 @@
       <sz val="8"/>
       <name val="맑은 고딕"/>
       <family val="2"/>
-      <charset val="129"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="맑은 고딕"/>
-      <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
@@ -1065,7 +1043,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1080,18 +1058,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1108,10 +1074,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1431,432 +1393,145 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E00837D9-2DC1-4B6E-B21E-25643E1A5509}">
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.75" customWidth="1"/>
     <col min="2" max="2" width="78.875" customWidth="1"/>
-    <col min="3" max="3" width="17.5" customWidth="1"/>
-    <col min="4" max="4" width="16.25" customWidth="1"/>
+    <col min="3" max="3" width="16.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>69</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C1" s="5"/>
-      <c r="D1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="33" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="33" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>146</v>
+        <v>115</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="C2" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="D2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>147</v>
+        <v>116</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="4"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C3" s="4"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>148</v>
+        <v>117</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="4"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C4" s="4"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>149</v>
+        <v>118</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="4"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C5" s="4"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>150</v>
+        <v>119</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="4"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C6" s="4"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>151</v>
+        <v>120</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="C7" s="7"/>
-      <c r="D7" s="4"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C7" s="4"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>152</v>
+        <v>121</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="C8" s="7"/>
-      <c r="D8" s="4"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C8" s="4"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>153</v>
+        <v>122</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="C9" s="7"/>
-      <c r="D9" s="4"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C9" s="4"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>80</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="C10" s="7"/>
-      <c r="D10" s="4"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C10" s="4"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="C11" s="4"/>
+    </row>
+    <row r="12" spans="1:3" ht="33" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="C11" s="7"/>
-      <c r="D11" s="4"/>
-    </row>
-    <row r="12" spans="1:4" ht="33" x14ac:dyDescent="0.3">
-      <c r="A12" s="3" t="s">
+      <c r="C12" s="4"/>
+    </row>
+    <row r="13" spans="1:3" ht="33" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="C13" s="4"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="C12" s="7"/>
-      <c r="D12" s="4"/>
-    </row>
-    <row r="13" spans="1:4" ht="33" x14ac:dyDescent="0.3">
-      <c r="A13" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="C13" s="7"/>
-      <c r="D13" s="4"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="C14" s="7"/>
-      <c r="D14" s="4"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="C15" s="7"/>
-      <c r="D15" s="3" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="C16" s="7"/>
-      <c r="D16" s="4"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="C17" s="7"/>
-      <c r="D17" s="4"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="C18" s="7"/>
-      <c r="D18" s="4"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="C19" s="7"/>
-      <c r="D19" s="4"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="C20" s="7"/>
-      <c r="D20" s="4"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="C21" s="7"/>
-      <c r="D21" s="4"/>
-    </row>
-    <row r="22" spans="1:4" ht="33" x14ac:dyDescent="0.3">
-      <c r="A22" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="C22" s="7"/>
-      <c r="D22" s="4"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="C23" s="7"/>
-      <c r="D23" s="4"/>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="C24" s="7"/>
-      <c r="D24" s="4"/>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="C25" s="7"/>
-      <c r="D25" s="4"/>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="C26" s="8" t="s">
-        <v>145</v>
-      </c>
-      <c r="D26" s="4"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="C27" s="7"/>
-      <c r="D27" s="4"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="C28" s="7"/>
-      <c r="D28" s="3" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="C29" s="7"/>
-      <c r="D29" s="4"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="C30" s="7"/>
-      <c r="D30" s="4"/>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A31" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="C31" s="7"/>
-      <c r="D31" s="4"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A32" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="C32" s="7"/>
-      <c r="D32" s="4"/>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A33" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="C33" s="7"/>
-      <c r="D33" s="4"/>
-    </row>
-    <row r="34" spans="1:4" ht="33" x14ac:dyDescent="0.3">
-      <c r="A34" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="C34" s="7"/>
-      <c r="D34" s="4"/>
-    </row>
-    <row r="35" spans="1:4" ht="33" x14ac:dyDescent="0.3">
-      <c r="A35" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="C35" s="7"/>
-      <c r="D35" s="4"/>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A36" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="C36" s="7"/>
-      <c r="D36" s="4"/>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A37" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="C37" s="7"/>
-      <c r="D37" s="4"/>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A38" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="C38" s="7"/>
-      <c r="D38" s="4"/>
-    </row>
-    <row r="39" spans="1:4" ht="33" x14ac:dyDescent="0.3">
-      <c r="A39" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="B39" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="C39" s="7"/>
-      <c r="D39" s="4"/>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A40" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="B40" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="C40" s="7"/>
-      <c r="D40" s="4"/>
+      <c r="C14" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="C2:C25"/>
-    <mergeCell ref="C26:C40"/>
-  </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
@@ -1864,6 +1539,300 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E899DD7E-A23D-4773-A976-7147E230A909}">
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.75" customWidth="1"/>
+    <col min="2" max="2" width="78.875" customWidth="1"/>
+    <col min="3" max="3" width="16.25" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C3" s="4"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C4" s="4"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="C5" s="4"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C6" s="4"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C7" s="4"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C8" s="4"/>
+    </row>
+    <row r="9" spans="1:3" ht="33" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C9" s="4"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C10" s="4"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C11" s="4"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="C12" s="4"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="C13" s="4"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C14" s="4"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3C55F7D-F09C-4C11-8F9D-6B95CD0841D9}">
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.75" customWidth="1"/>
+    <col min="2" max="2" width="78.875" customWidth="1"/>
+    <col min="3" max="3" width="16.25" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C3" s="4"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="C4" s="4"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C5" s="4"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="C6" s="4"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C7" s="4"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="C8" s="4"/>
+    </row>
+    <row r="9" spans="1:3" ht="33" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C9" s="4"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="C10" s="4"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C11" s="4"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C12" s="4"/>
+    </row>
+    <row r="13" spans="1:3" ht="33" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C13" s="4"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="C14" s="4"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5D53722-342C-4F1F-B5E5-00FB61208351}">
   <dimension ref="A1:C32"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>

</xml_diff>